<commit_message>
Add new error analyzer
</commit_message>
<xml_diff>
--- a/benchmark_reports/benchmark_comparison.xlsx
+++ b/benchmark_reports/benchmark_comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,30 +454,25 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>LLM Correctness</t>
+          <t>False Refusal</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>False Refusal</t>
+          <t>Correct Refusal</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Correct Refusal</t>
+          <t>Hallucination</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Hallucination</t>
+          <t>Latency (s)</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
-        <is>
-          <t>Latency (s)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
         <is>
           <t>Throughput (samples/s)</t>
         </is>
@@ -500,34 +495,31 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14.4186</v>
+        <v>13.4884</v>
       </c>
       <c r="E2" t="n">
-        <v>63.8711</v>
+        <v>62.9408</v>
       </c>
       <c r="F2" t="n">
-        <v>61.7956</v>
+        <v>60.8653</v>
       </c>
       <c r="G2" t="n">
         <v>34.5178</v>
       </c>
       <c r="H2" t="n">
-        <v>91.81399999999999</v>
+        <v>0.5076000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7614</v>
+        <v>61.1111</v>
       </c>
       <c r="J2" t="n">
-        <v>72.2222</v>
+        <v>22.2222</v>
       </c>
       <c r="K2" t="n">
-        <v>22.2222</v>
+        <v>0.0483</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0483</v>
-      </c>
-      <c r="M2" t="n">
-        <v>20.6827</v>
+        <v>20.7051</v>
       </c>
     </row>
     <row r="3">
@@ -547,34 +539,31 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>18.1395</v>
+        <v>17.907</v>
       </c>
       <c r="E3" t="n">
-        <v>61.4464</v>
+        <v>61.2138</v>
       </c>
       <c r="F3" t="n">
-        <v>60.6432</v>
+        <v>60.4106</v>
       </c>
       <c r="G3" t="n">
         <v>36.5482</v>
       </c>
       <c r="H3" t="n">
-        <v>86.5814</v>
+        <v>1.0152</v>
       </c>
       <c r="I3" t="n">
-        <v>1.7766</v>
+        <v>88.88890000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>91.66670000000001</v>
+        <v>5.5556</v>
       </c>
       <c r="K3" t="n">
-        <v>8.333299999999999</v>
+        <v>0.0211</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0211</v>
-      </c>
-      <c r="M3" t="n">
-        <v>47.3595</v>
+        <v>47.2815</v>
       </c>
     </row>
     <row r="4">
@@ -594,34 +583,31 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19.5349</v>
+        <v>19.3023</v>
       </c>
       <c r="E4" t="n">
-        <v>67.4823</v>
+        <v>67.24979999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>66.19159999999999</v>
+        <v>65.959</v>
       </c>
       <c r="G4" t="n">
         <v>42.3858</v>
       </c>
       <c r="H4" t="n">
-        <v>88.3488</v>
+        <v>2.0305</v>
       </c>
       <c r="I4" t="n">
-        <v>3.0457</v>
+        <v>91.66670000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>94.4444</v>
+        <v>5.5556</v>
       </c>
       <c r="K4" t="n">
-        <v>5.5556</v>
+        <v>0.0287</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0285</v>
-      </c>
-      <c r="M4" t="n">
-        <v>35.0524</v>
+        <v>34.8797</v>
       </c>
     </row>
     <row r="5">
@@ -653,22 +639,19 @@
         <v>40.8629</v>
       </c>
       <c r="H5" t="n">
-        <v>87.97669999999999</v>
+        <v>1.7766</v>
       </c>
       <c r="I5" t="n">
-        <v>2.2843</v>
+        <v>91.66670000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>91.66670000000001</v>
+        <v>2.7778</v>
       </c>
       <c r="K5" t="n">
-        <v>5.5556</v>
+        <v>0.0281</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0281</v>
-      </c>
-      <c r="M5" t="n">
-        <v>35.5297</v>
+        <v>35.5636</v>
       </c>
     </row>
     <row r="6">
@@ -688,34 +671,31 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18.8372</v>
+        <v>18.6047</v>
       </c>
       <c r="E6" t="n">
-        <v>66.32470000000001</v>
+        <v>66.09220000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>65.15519999999999</v>
+        <v>64.9226</v>
       </c>
       <c r="G6" t="n">
         <v>40.3553</v>
       </c>
       <c r="H6" t="n">
-        <v>88.02330000000001</v>
+        <v>1.7766</v>
       </c>
       <c r="I6" t="n">
-        <v>3.0457</v>
+        <v>91.66670000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>94.4444</v>
+        <v>5.5556</v>
       </c>
       <c r="K6" t="n">
-        <v>5.5556</v>
+        <v>0.0281</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0282</v>
-      </c>
-      <c r="M6" t="n">
-        <v>35.4399</v>
+        <v>35.5353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update visualization for model configuration results
</commit_message>
<xml_diff>
--- a/benchmark_reports/benchmark_comparison.xlsx
+++ b/benchmark_reports/benchmark_comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,95 +481,95 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Qwen3-VL-4B-Instruct</t>
+          <t>qwen3_examassist_merged_4b_qlora_domain</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>QLoRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>r=8</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>13.4884</v>
+        <v>17.907</v>
       </c>
       <c r="E2" t="n">
-        <v>62.9408</v>
+        <v>61.2138</v>
       </c>
       <c r="F2" t="n">
-        <v>60.8653</v>
+        <v>60.4106</v>
       </c>
       <c r="G2" t="n">
-        <v>34.5178</v>
+        <v>36.5482</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5076000000000001</v>
+        <v>1.0152</v>
       </c>
       <c r="I2" t="n">
-        <v>61.1111</v>
+        <v>88.88890000000001</v>
       </c>
       <c r="J2" t="n">
-        <v>22.2222</v>
+        <v>5.5556</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0483</v>
+        <v>0.0211</v>
       </c>
       <c r="L2" t="n">
-        <v>20.7051</v>
+        <v>47.2815</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>qwen3_examassist_merged_4b_qlora_domain</t>
+          <t>qwen3_examassist_merged_4b_rslora_domain_v5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>QLoRA</t>
+          <t>RSLoRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>r=8</t>
+          <t>r=16</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>17.907</v>
+        <v>18.6047</v>
       </c>
       <c r="E3" t="n">
-        <v>61.2138</v>
+        <v>66.09220000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>60.4106</v>
+        <v>64.9226</v>
       </c>
       <c r="G3" t="n">
-        <v>36.5482</v>
+        <v>40.3553</v>
       </c>
       <c r="H3" t="n">
-        <v>1.0152</v>
+        <v>1.7766</v>
       </c>
       <c r="I3" t="n">
-        <v>88.88890000000001</v>
+        <v>91.66670000000001</v>
       </c>
       <c r="J3" t="n">
         <v>5.5556</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0211</v>
+        <v>0.0281</v>
       </c>
       <c r="L3" t="n">
-        <v>47.2815</v>
+        <v>35.5353</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>qwen3_examassist_merged_4b_rslora_domain_v5</t>
+          <t>qwen3_examassist_merged_4b_rslora_domain_v4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -579,20 +579,20 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>r=16</t>
+          <t>r=32</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.6047</v>
+        <v>18.8372</v>
       </c>
       <c r="E4" t="n">
-        <v>66.09220000000001</v>
+        <v>65.9006</v>
       </c>
       <c r="F4" t="n">
-        <v>64.9226</v>
+        <v>64.41200000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>40.3553</v>
+        <v>40.8629</v>
       </c>
       <c r="H4" t="n">
         <v>1.7766</v>
@@ -601,19 +601,19 @@
         <v>91.66670000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>5.5556</v>
+        <v>2.7778</v>
       </c>
       <c r="K4" t="n">
         <v>0.0281</v>
       </c>
       <c r="L4" t="n">
-        <v>35.5353</v>
+        <v>35.5636</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>qwen3_examassist_merged_4b_rslora_domain_v4</t>
+          <t>qwen3_examassist_merged_4b_rslora_domain_v3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -623,78 +623,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>r=32</t>
+          <t>r=8</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18.8372</v>
+        <v>19.3023</v>
       </c>
       <c r="E5" t="n">
-        <v>65.9006</v>
+        <v>67.24979999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>64.41200000000001</v>
+        <v>65.959</v>
       </c>
       <c r="G5" t="n">
-        <v>40.8629</v>
+        <v>42.3858</v>
       </c>
       <c r="H5" t="n">
-        <v>1.7766</v>
+        <v>2.0305</v>
       </c>
       <c r="I5" t="n">
         <v>91.66670000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>2.7778</v>
+        <v>5.5556</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0281</v>
+        <v>0.0287</v>
       </c>
       <c r="L5" t="n">
-        <v>35.5636</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>qwen3_examassist_merged_4b_rslora_domain_v3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>RSLoRA</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>r=8</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>19.3023</v>
-      </c>
-      <c r="E6" t="n">
-        <v>67.24979999999999</v>
-      </c>
-      <c r="F6" t="n">
-        <v>65.959</v>
-      </c>
-      <c r="G6" t="n">
-        <v>42.3858</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2.0305</v>
-      </c>
-      <c r="I6" t="n">
-        <v>91.66670000000001</v>
-      </c>
-      <c r="J6" t="n">
-        <v>5.5556</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.0287</v>
-      </c>
-      <c r="L6" t="n">
         <v>34.8797</v>
       </c>
     </row>

</xml_diff>